<commit_message>
Contributo Caldaia come voce dedicata nel confronto e nell'esportazione Excel
</commit_message>
<xml_diff>
--- a/tariffe/2026-09/residenziale/tariffe_illumia_template.xlsx
+++ b/tariffe/2026-09/residenziale/tariffe_illumia_template.xlsx
@@ -10,7 +10,7 @@
     <sheet name="tariffe" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'tariffe'!$A$1:$M$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'tariffe'!$A$1:$M$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M24"/>
+  <dimension ref="A1:M25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1833,12 +1833,12 @@
         </is>
       </c>
       <c r="J24" s="2" t="n">
-        <v>226.8</v>
+        <v>144</v>
       </c>
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>Da PDF CE-ILLUMIA-CALDAIA-A-MODO-TUO-FIX-GAS-36: corrispettivo annuo 144 €/PdR/anno + 6,90 €/mese per 24 mesi (82,80 €/anno)</t>
+          <t>Da PDF CE-ILLUMIA-CALDAIA-A-MODO-TUO-FIX-GAS-36: corrispettivo annuo 144 €/PdR/anno</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
@@ -1847,8 +1847,65 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>ILLUMIA</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>RESIDENZIALE</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>FISSA</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>CALDAIA A MODO TUO FIX GAS 36</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>46276</v>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>quota_mensile_extra</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>€/mese</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Da PDF CE-ILLUMIA-CALDAIA-A-MODO-TUO-FIX-GAS-36: corrispettivo pari a 6,90 €/mese per 24 mesi</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M24"/>
+  <autoFilter ref="A1:M25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>